<commit_message>
Improved final proposal handling with specsheets
</commit_message>
<xml_diff>
--- a/src/templates/settings.xlsx
+++ b/src/templates/settings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joseph\Desktop\Code\MSSProposalAutomation\src\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DC65282-043D-4087-86E6-9BAE3307C2E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2DBB867-21B4-4E0A-B25A-C40D4B9B6D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" activeTab="3" xr2:uid="{33255D11-AE72-42F8-B637-887034ED5189}"/>
+    <workbookView xWindow="2057" yWindow="3969" windowWidth="15514" windowHeight="10740" activeTab="2" xr2:uid="{33255D11-AE72-42F8-B637-887034ED5189}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="76">
   <si>
     <t>Aliases</t>
   </si>
@@ -234,6 +234,42 @@
   </si>
   <si>
     <t>B20</t>
+  </si>
+  <si>
+    <t>Dedicated Subpanel (Critical Loads Backup) for Off-Grid use:</t>
+  </si>
+  <si>
+    <t>{{OFF_GRID_SUBPANEL_OMIT}}</t>
+  </si>
+  <si>
+    <t>{{OFF_GRID_SUBPANEL_OPTION}}</t>
+  </si>
+  <si>
+    <t>Omit Dedicated Subpanel (On-Grid Only): Subtract</t>
+  </si>
+  <si>
+    <t>{{UTILITY_LINK_MID}}</t>
+  </si>
+  <si>
+    <t>https://www.mid.org/saving-energy-money/solar/</t>
+  </si>
+  <si>
+    <t>{{UTILITY_LINK_PGE}}</t>
+  </si>
+  <si>
+    <t>https://www.pge.com/en/clean-energy/solar/getting-started-with-solar/solar-billing-plan.html#residential/</t>
+  </si>
+  <si>
+    <t>Inverter Efficiency</t>
+  </si>
+  <si>
+    <t>B21</t>
+  </si>
+  <si>
+    <t>{{APPLICATION_FEE_MID}}</t>
+  </si>
+  <si>
+    <t>{{APPLICATION_FEE_PGE}}</t>
   </si>
 </sst>
 </file>
@@ -282,10 +318,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -620,7 +659,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B33C8AC-ACEE-433F-A601-64D42BCBF1D1}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40.69140625" style="2" bestFit="1" customWidth="1"/>
@@ -698,6 +737,54 @@
       </c>
       <c r="B9" s="2" t="s">
         <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" s="3">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B15" s="3">
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -831,10 +918,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A703C62-77F3-49A3-80D8-DCD51CDBB0B7}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.4609375" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.07421875" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="16384" width="9.23046875" style="2"/>
   </cols>
   <sheetData>
@@ -848,6 +935,14 @@
         <v>10</v>
       </c>
       <c r="B2" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="2">
         <v>3</v>
       </c>
     </row>
@@ -858,7 +953,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F51E514D-75A4-472E-97C1-71E280C73026}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.765625" style="2" bestFit="1" customWidth="1"/>
@@ -943,6 +1038,14 @@
         <v>63</v>
       </c>
     </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>